<commit_message>
Health mal wieder laufen lassen. Secrets jetzt aus Config
</commit_message>
<xml_diff>
--- a/docs/Health vs Fitibit.xlsx
+++ b/docs/Health vs Fitibit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\permi\git\ThosSuite\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98499E3-9977-4A0B-89F1-046C392757B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF1C7ED-7858-4BAB-8A5E-93DAAAB7F48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{75A032EB-1DBF-418D-AE42-777C8ACB1553}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -126,12 +126,12 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -157,79 +157,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -543,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B59795-D574-4235-A884-9D5CA251F90A}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
@@ -595,7 +522,7 @@
         <v>14971</v>
       </c>
       <c r="H2" s="4">
-        <f>B2/G2</f>
+        <f t="shared" ref="H2:H32" si="0">B2/G2</f>
         <v>0.98189833678444993</v>
       </c>
     </row>
@@ -622,7 +549,7 @@
         <v>4811</v>
       </c>
       <c r="H3" s="4">
-        <f>B3/G3</f>
+        <f t="shared" si="0"/>
         <v>0.9669507378923301</v>
       </c>
     </row>
@@ -649,7 +576,7 @@
         <v>11884</v>
       </c>
       <c r="H4" s="4">
-        <f>B4/G4</f>
+        <f t="shared" si="0"/>
         <v>0.99318411309323462</v>
       </c>
     </row>
@@ -676,7 +603,7 @@
         <v>8887</v>
       </c>
       <c r="H5" s="4">
-        <f>B5/G5</f>
+        <f t="shared" si="0"/>
         <v>0.97333183301451554</v>
       </c>
     </row>
@@ -703,7 +630,7 @@
         <v>11686</v>
       </c>
       <c r="H6" s="4">
-        <f>B6/G6</f>
+        <f t="shared" si="0"/>
         <v>0.9803183296251925</v>
       </c>
     </row>
@@ -730,7 +657,7 @@
         <v>6995</v>
       </c>
       <c r="H7" s="4">
-        <f>B7/G7</f>
+        <f t="shared" si="0"/>
         <v>0.99814152966404579</v>
       </c>
     </row>
@@ -757,7 +684,7 @@
         <v>10286</v>
       </c>
       <c r="H8" s="4">
-        <f>B8/G8</f>
+        <f t="shared" si="0"/>
         <v>0.99834726813144081</v>
       </c>
     </row>
@@ -784,7 +711,7 @@
         <v>12402</v>
       </c>
       <c r="H9" s="4">
-        <f>B9/G9</f>
+        <f t="shared" si="0"/>
         <v>0.99943557490727297</v>
       </c>
     </row>
@@ -811,7 +738,7 @@
         <v>12098</v>
       </c>
       <c r="H10" s="4">
-        <f>B10/G10</f>
+        <f t="shared" si="0"/>
         <v>0.99057695486857333</v>
       </c>
     </row>
@@ -838,7 +765,7 @@
         <v>11905</v>
       </c>
       <c r="H11" s="4">
-        <f>B11/G11</f>
+        <f t="shared" si="0"/>
         <v>0.98362032759344808</v>
       </c>
     </row>
@@ -865,7 +792,7 @@
         <v>9259</v>
       </c>
       <c r="H12" s="4">
-        <f>B12/G12</f>
+        <f t="shared" si="0"/>
         <v>0.98876768549519389</v>
       </c>
     </row>
@@ -892,7 +819,7 @@
         <v>15198</v>
       </c>
       <c r="H13" s="4">
-        <f>B13/G13</f>
+        <f t="shared" si="0"/>
         <v>0.9940781681800237</v>
       </c>
     </row>
@@ -919,7 +846,7 @@
         <v>11523</v>
       </c>
       <c r="H14" s="4">
-        <f>B14/G14</f>
+        <f t="shared" si="0"/>
         <v>0.9903670919031502</v>
       </c>
     </row>
@@ -946,7 +873,7 @@
         <v>6396</v>
       </c>
       <c r="H15" s="4">
-        <f>B15/G15</f>
+        <f t="shared" si="0"/>
         <v>0.97967479674796742</v>
       </c>
     </row>
@@ -973,7 +900,7 @@
         <v>10552</v>
       </c>
       <c r="H16" s="4">
-        <f>B16/G16</f>
+        <f t="shared" si="0"/>
         <v>0.98815390447308571</v>
       </c>
     </row>
@@ -1000,7 +927,7 @@
         <v>13170</v>
       </c>
       <c r="H17" s="4">
-        <f>B17/G17</f>
+        <f t="shared" si="0"/>
         <v>0.98352315869400153</v>
       </c>
     </row>
@@ -1027,7 +954,7 @@
         <v>17013</v>
       </c>
       <c r="H18" s="4">
-        <f>B18/G18</f>
+        <f t="shared" si="0"/>
         <v>0.98959619114794573</v>
       </c>
     </row>
@@ -1054,7 +981,7 @@
         <v>12659</v>
       </c>
       <c r="H19" s="4">
-        <f>B19/G19</f>
+        <f t="shared" si="0"/>
         <v>0.99210048187060584</v>
       </c>
     </row>
@@ -1081,7 +1008,7 @@
         <v>11357</v>
       </c>
       <c r="H20" s="4">
-        <f>B20/G20</f>
+        <f t="shared" si="0"/>
         <v>1.001320771330457</v>
       </c>
       <c r="I20" t="s">
@@ -1111,7 +1038,7 @@
         <v>6420</v>
       </c>
       <c r="H21" s="4">
-        <f>B21/G21</f>
+        <f t="shared" si="0"/>
         <v>0.98551401869158883</v>
       </c>
     </row>
@@ -1138,7 +1065,7 @@
         <v>9941</v>
       </c>
       <c r="H22" s="4">
-        <f>B22/G22</f>
+        <f t="shared" si="0"/>
         <v>0.99557388592696916</v>
       </c>
     </row>
@@ -1165,7 +1092,7 @@
         <v>11771</v>
       </c>
       <c r="H23" s="4">
-        <f>B23/G23</f>
+        <f t="shared" si="0"/>
         <v>0.98708690850395042</v>
       </c>
     </row>
@@ -1192,7 +1119,7 @@
         <v>12200</v>
       </c>
       <c r="H24" s="4">
-        <f>B24/G24</f>
+        <f t="shared" si="0"/>
         <v>1.0200819672131147</v>
       </c>
     </row>
@@ -1219,7 +1146,7 @@
         <v>10159</v>
       </c>
       <c r="H25" s="4">
-        <f>B25/G25</f>
+        <f t="shared" si="0"/>
         <v>0.99015651146766415</v>
       </c>
     </row>
@@ -1246,7 +1173,7 @@
         <v>8472</v>
       </c>
       <c r="H26" s="4">
-        <f>B26/G26</f>
+        <f t="shared" si="0"/>
         <v>1.0243153918791312</v>
       </c>
     </row>
@@ -1273,7 +1200,7 @@
         <v>15682</v>
       </c>
       <c r="H27" s="4">
-        <f>B27/G27</f>
+        <f t="shared" si="0"/>
         <v>0.99853335033796708</v>
       </c>
     </row>
@@ -1300,7 +1227,7 @@
         <v>11970</v>
       </c>
       <c r="H28" s="4">
-        <f>B28/G28</f>
+        <f t="shared" si="0"/>
         <v>1.005764411027569</v>
       </c>
     </row>
@@ -1327,7 +1254,7 @@
         <v>9834</v>
       </c>
       <c r="H29" s="4">
-        <f>B29/G29</f>
+        <f t="shared" si="0"/>
         <v>0.99877974374618672</v>
       </c>
     </row>
@@ -1354,7 +1281,7 @@
         <v>11152</v>
       </c>
       <c r="H30" s="4">
-        <f>B30/G30</f>
+        <f t="shared" si="0"/>
         <v>1.0148852223816356</v>
       </c>
     </row>
@@ -1381,7 +1308,7 @@
         <v>13588</v>
       </c>
       <c r="H31" s="4">
-        <f>B31/G31</f>
+        <f t="shared" si="0"/>
         <v>1.0236237856932588</v>
       </c>
     </row>
@@ -1408,7 +1335,7 @@
         <v>12214</v>
       </c>
       <c r="H32" s="4">
-        <f>B32/G32</f>
+        <f t="shared" si="0"/>
         <v>0.98976584247584742</v>
       </c>
     </row>
@@ -1435,7 +1362,7 @@
         <v>10356</v>
       </c>
       <c r="H33" s="4">
-        <f t="shared" ref="H33:H35" si="0">B33/G33</f>
+        <f t="shared" ref="H33:H60" si="1">B33/G33</f>
         <v>1.0085940517574352</v>
       </c>
     </row>
@@ -1462,7 +1389,7 @@
         <v>12301</v>
       </c>
       <c r="H34" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.99991870579627673</v>
       </c>
     </row>
@@ -1489,17 +1416,700 @@
         <v>10587</v>
       </c>
       <c r="H35" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.0421271370548786</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>46208</v>
+      </c>
+      <c r="B36" s="2">
+        <v>10196</v>
+      </c>
+      <c r="C36" s="2">
+        <v>10196</v>
+      </c>
+      <c r="D36" s="2">
+        <v>12574</v>
+      </c>
+      <c r="E36" s="2">
+        <v>10432</v>
+      </c>
+      <c r="F36" s="2">
+        <v>10432</v>
+      </c>
+      <c r="G36" s="2">
+        <v>10432</v>
+      </c>
+      <c r="H36" s="4">
+        <f t="shared" si="1"/>
+        <v>0.97737730061349692</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>46209</v>
+      </c>
+      <c r="B37" s="2">
+        <v>7391</v>
+      </c>
+      <c r="C37" s="2">
+        <v>7391</v>
+      </c>
+      <c r="D37" s="2">
+        <v>7391</v>
+      </c>
+      <c r="E37" s="2">
+        <v>7397</v>
+      </c>
+      <c r="F37" s="2">
+        <v>7397</v>
+      </c>
+      <c r="G37" s="2">
+        <v>7397</v>
+      </c>
+      <c r="H37" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99918886034879006</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>46210</v>
+      </c>
+      <c r="B38" s="2">
+        <v>9432</v>
+      </c>
+      <c r="C38" s="2">
+        <v>9432</v>
+      </c>
+      <c r="D38" s="2">
+        <v>9432</v>
+      </c>
+      <c r="E38" s="2">
+        <v>9595</v>
+      </c>
+      <c r="F38" s="2">
+        <v>9595</v>
+      </c>
+      <c r="G38" s="2">
+        <v>9595</v>
+      </c>
+      <c r="H38" s="4">
+        <f t="shared" si="1"/>
+        <v>0.9830119854090672</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>46211</v>
+      </c>
+      <c r="B39" s="2">
+        <v>11937</v>
+      </c>
+      <c r="C39" s="2">
+        <v>11937</v>
+      </c>
+      <c r="D39" s="2">
+        <v>11937</v>
+      </c>
+      <c r="E39" s="2">
+        <v>11974</v>
+      </c>
+      <c r="F39" s="2">
+        <v>11974</v>
+      </c>
+      <c r="G39" s="2">
+        <v>11974</v>
+      </c>
+      <c r="H39" s="4">
+        <f t="shared" si="1"/>
+        <v>0.9969099716051445</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>46212</v>
+      </c>
+      <c r="B40" s="2">
+        <v>11638</v>
+      </c>
+      <c r="C40" s="2">
+        <v>11638</v>
+      </c>
+      <c r="D40" s="2">
+        <v>11638</v>
+      </c>
+      <c r="E40" s="2">
+        <v>11738</v>
+      </c>
+      <c r="F40" s="2">
+        <v>11738</v>
+      </c>
+      <c r="G40" s="2">
+        <v>11738</v>
+      </c>
+      <c r="H40" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99148066110069855</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>46213</v>
+      </c>
+      <c r="B41" s="2">
+        <v>11122</v>
+      </c>
+      <c r="C41" s="2">
+        <v>11122</v>
+      </c>
+      <c r="D41" s="2">
+        <v>11122</v>
+      </c>
+      <c r="E41" s="2">
+        <v>11215</v>
+      </c>
+      <c r="F41" s="2">
+        <v>11215</v>
+      </c>
+      <c r="G41" s="2">
+        <v>11215</v>
+      </c>
+      <c r="H41" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99170753455193938</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>46214</v>
+      </c>
+      <c r="B42" s="2">
+        <v>7833</v>
+      </c>
+      <c r="C42" s="2">
+        <v>7833</v>
+      </c>
+      <c r="D42" s="2">
+        <v>7833</v>
+      </c>
+      <c r="E42" s="2">
+        <v>7885</v>
+      </c>
+      <c r="F42" s="2">
+        <v>7885</v>
+      </c>
+      <c r="G42" s="2">
+        <v>7885</v>
+      </c>
+      <c r="H42" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99340519974635388</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
+        <v>46215</v>
+      </c>
+      <c r="B43" s="2">
+        <v>16760</v>
+      </c>
+      <c r="C43" s="2">
+        <v>16760</v>
+      </c>
+      <c r="D43" s="2">
+        <v>16760</v>
+      </c>
+      <c r="E43" s="2">
+        <v>16925</v>
+      </c>
+      <c r="F43" s="2">
+        <v>16925</v>
+      </c>
+      <c r="G43" s="2">
+        <v>16925</v>
+      </c>
+      <c r="H43" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99025110782865589</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
+        <v>46216</v>
+      </c>
+      <c r="B44" s="2">
+        <v>7355</v>
+      </c>
+      <c r="C44" s="2">
+        <v>7355</v>
+      </c>
+      <c r="D44" s="2">
+        <v>7355</v>
+      </c>
+      <c r="E44" s="2">
+        <v>7417</v>
+      </c>
+      <c r="F44" s="2">
+        <v>7417</v>
+      </c>
+      <c r="G44" s="2">
+        <v>7417</v>
+      </c>
+      <c r="H44" s="4">
+        <f t="shared" si="1"/>
+        <v>0.9916408251314548</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="3">
+        <v>46217</v>
+      </c>
+      <c r="B45" s="2">
+        <v>12108</v>
+      </c>
+      <c r="C45" s="2">
+        <v>12108</v>
+      </c>
+      <c r="D45" s="2">
+        <v>12108</v>
+      </c>
+      <c r="E45" s="2">
+        <v>12156</v>
+      </c>
+      <c r="F45" s="2">
+        <v>12156</v>
+      </c>
+      <c r="G45" s="2">
+        <v>12156</v>
+      </c>
+      <c r="H45" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99605133267522217</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="3">
+        <v>46218</v>
+      </c>
+      <c r="B46" s="2">
+        <v>9290</v>
+      </c>
+      <c r="C46" s="2">
+        <v>9290</v>
+      </c>
+      <c r="D46" s="2">
+        <v>9290</v>
+      </c>
+      <c r="E46" s="2">
+        <v>9290</v>
+      </c>
+      <c r="F46" s="2">
+        <v>9290</v>
+      </c>
+      <c r="G46" s="2">
+        <v>9290</v>
+      </c>
+      <c r="H46" s="4">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="3">
+        <v>46219</v>
+      </c>
+      <c r="B47" s="2">
+        <v>13223</v>
+      </c>
+      <c r="C47" s="2">
+        <v>13223</v>
+      </c>
+      <c r="D47" s="2">
+        <v>13223</v>
+      </c>
+      <c r="E47" s="2">
+        <v>13247</v>
+      </c>
+      <c r="F47" s="2">
+        <v>13247</v>
+      </c>
+      <c r="G47" s="2">
+        <v>13247</v>
+      </c>
+      <c r="H47" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99818826904204727</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="3">
+        <v>46220</v>
+      </c>
+      <c r="B48" s="2">
+        <v>16621</v>
+      </c>
+      <c r="C48" s="2">
+        <v>16621</v>
+      </c>
+      <c r="D48" s="2">
+        <v>16621</v>
+      </c>
+      <c r="E48" s="2">
+        <v>16770</v>
+      </c>
+      <c r="F48" s="2">
+        <v>16770</v>
+      </c>
+      <c r="G48" s="2">
+        <v>16770</v>
+      </c>
+      <c r="H48" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99111508646392366</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="3">
+        <v>46221</v>
+      </c>
+      <c r="B49" s="2">
+        <v>11917</v>
+      </c>
+      <c r="C49" s="2">
+        <v>11917</v>
+      </c>
+      <c r="D49" s="2">
+        <v>11917</v>
+      </c>
+      <c r="E49" s="2">
+        <v>12090</v>
+      </c>
+      <c r="F49" s="2">
+        <v>12090</v>
+      </c>
+      <c r="G49" s="2">
+        <v>12090</v>
+      </c>
+      <c r="H49" s="4">
+        <f t="shared" si="1"/>
+        <v>0.98569065343258888</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="3">
+        <v>46222</v>
+      </c>
+      <c r="B50" s="2">
+        <v>11235</v>
+      </c>
+      <c r="C50" s="2">
+        <v>11235</v>
+      </c>
+      <c r="D50" s="2">
+        <v>11235</v>
+      </c>
+      <c r="E50" s="2">
+        <v>11407</v>
+      </c>
+      <c r="F50" s="2">
+        <v>11407</v>
+      </c>
+      <c r="G50" s="2">
+        <v>11407</v>
+      </c>
+      <c r="H50" s="4">
+        <f t="shared" si="1"/>
+        <v>0.9849215394056281</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A51" s="3">
+        <v>46223</v>
+      </c>
+      <c r="B51" s="2">
+        <v>13914</v>
+      </c>
+      <c r="C51" s="2">
+        <v>13914</v>
+      </c>
+      <c r="D51" s="2">
+        <v>13914</v>
+      </c>
+      <c r="E51" s="2">
+        <v>14037</v>
+      </c>
+      <c r="F51" s="2">
+        <v>14037</v>
+      </c>
+      <c r="G51" s="2">
+        <v>14037</v>
+      </c>
+      <c r="H51" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99123744389826884</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A52" s="3">
+        <v>46224</v>
+      </c>
+      <c r="B52" s="2">
+        <v>20663</v>
+      </c>
+      <c r="C52" s="2">
+        <v>20663</v>
+      </c>
+      <c r="D52" s="2">
+        <v>20663</v>
+      </c>
+      <c r="E52" s="2">
+        <v>20863</v>
+      </c>
+      <c r="F52" s="2">
+        <v>20863</v>
+      </c>
+      <c r="G52" s="2">
+        <v>20863</v>
+      </c>
+      <c r="H52" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99041365096103151</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="3">
+        <v>46225</v>
+      </c>
+      <c r="B53" s="2">
+        <v>27266</v>
+      </c>
+      <c r="C53" s="2">
+        <v>27266</v>
+      </c>
+      <c r="D53" s="2">
+        <v>27266</v>
+      </c>
+      <c r="E53" s="2">
+        <v>27552</v>
+      </c>
+      <c r="F53" s="2">
+        <v>27552</v>
+      </c>
+      <c r="G53" s="2">
+        <v>27552</v>
+      </c>
+      <c r="H53" s="4">
+        <f t="shared" si="1"/>
+        <v>0.98961962833914052</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="3">
+        <v>46226</v>
+      </c>
+      <c r="B54" s="2">
+        <v>29146</v>
+      </c>
+      <c r="C54" s="2">
+        <v>29120</v>
+      </c>
+      <c r="D54" s="2">
+        <v>29146</v>
+      </c>
+      <c r="E54" s="2">
+        <v>29480</v>
+      </c>
+      <c r="F54" s="2">
+        <v>29480</v>
+      </c>
+      <c r="G54" s="2">
+        <v>29480</v>
+      </c>
+      <c r="H54" s="4">
+        <f t="shared" si="1"/>
+        <v>0.9886702849389416</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="3">
+        <v>46227</v>
+      </c>
+      <c r="B55" s="2">
+        <v>7988</v>
+      </c>
+      <c r="C55" s="2">
+        <v>7988</v>
+      </c>
+      <c r="D55" s="2">
+        <v>7988</v>
+      </c>
+      <c r="E55" s="2">
+        <v>8215</v>
+      </c>
+      <c r="F55" s="2">
+        <v>8215</v>
+      </c>
+      <c r="G55" s="2">
+        <v>8215</v>
+      </c>
+      <c r="H55" s="4">
+        <f t="shared" si="1"/>
+        <v>0.97236762020693857</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="3">
+        <v>46228</v>
+      </c>
+      <c r="B56" s="2">
+        <v>5024</v>
+      </c>
+      <c r="C56" s="2">
+        <v>5024</v>
+      </c>
+      <c r="D56" s="2">
+        <v>5024</v>
+      </c>
+      <c r="E56" s="2">
+        <v>5076</v>
+      </c>
+      <c r="F56" s="2">
+        <v>5076</v>
+      </c>
+      <c r="G56" s="2">
+        <v>5076</v>
+      </c>
+      <c r="H56" s="4">
+        <f t="shared" si="1"/>
+        <v>0.98975571315996846</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="3">
+        <v>46229</v>
+      </c>
+      <c r="B57" s="2">
+        <v>4943</v>
+      </c>
+      <c r="C57" s="2">
+        <v>4943</v>
+      </c>
+      <c r="D57" s="2">
+        <v>4943</v>
+      </c>
+      <c r="E57" s="2">
+        <v>4959</v>
+      </c>
+      <c r="F57" s="2">
+        <v>4959</v>
+      </c>
+      <c r="G57" s="2">
+        <v>4959</v>
+      </c>
+      <c r="H57" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99677354305303489</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A58" s="3">
+        <v>46230</v>
+      </c>
+      <c r="B58" s="2">
+        <v>8996</v>
+      </c>
+      <c r="C58" s="2">
+        <v>8996</v>
+      </c>
+      <c r="D58" s="2">
+        <v>8996</v>
+      </c>
+      <c r="E58" s="2">
+        <v>8996</v>
+      </c>
+      <c r="F58" s="2">
+        <v>8996</v>
+      </c>
+      <c r="G58" s="2">
+        <v>8996</v>
+      </c>
+      <c r="H58" s="4">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="3">
+        <v>46231</v>
+      </c>
+      <c r="B59" s="2">
+        <v>10506</v>
+      </c>
+      <c r="C59" s="2">
+        <v>10506</v>
+      </c>
+      <c r="D59" s="2">
+        <v>10506</v>
+      </c>
+      <c r="E59" s="2">
+        <v>10669</v>
+      </c>
+      <c r="F59" s="2">
+        <v>10669</v>
+      </c>
+      <c r="G59" s="2">
+        <v>10669</v>
+      </c>
+      <c r="H59" s="4">
+        <f t="shared" si="1"/>
+        <v>0.98472209204236572</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="3">
+        <v>46232</v>
+      </c>
+      <c r="B60" s="2">
+        <v>9573</v>
+      </c>
+      <c r="C60" s="2">
+        <v>9573</v>
+      </c>
+      <c r="D60" s="2">
+        <v>9573</v>
+      </c>
+      <c r="E60" s="2">
+        <v>9599</v>
+      </c>
+      <c r="F60" s="2">
+        <v>9599</v>
+      </c>
+      <c r="G60" s="2">
+        <v>9599</v>
+      </c>
+      <c r="H60" s="4">
+        <f t="shared" si="1"/>
+        <v>0.99729138451922072</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:F35">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>B2&lt;&gt;$G2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>B2=$G2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B36:F60">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>B36&lt;&gt;$G36</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>B36=$G36</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>